<commit_message>
Add emails and explicit time-period labels to adoption workbook
Both tables now carry a "Time period: ALL TIME" header with the dashboard
date range, an Email column (TrueSeaMoss addresses included), a Platform
column, and footnotes on recent-window activity.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxMtvSYX4QyFmV6dcFDu1y
</commit_message>
<xml_diff>
--- a/iq_adoption_equipfoods_tsm.xlsx
+++ b/iq_adoption_equipfoods_tsm.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0;&quot;—&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,9 +35,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="004A3AB5"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -53,6 +53,12 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -99,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +116,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -117,6 +126,7 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,14 +492,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>iQ adoption by user — all-time. Excludes Equipfoods Pulse (analytics.saras@equipfoods.com).</t>
+          <t>Time period: ALL TIME (all available data — dashboard range May 3, 2026 – Sep 11, 2026)</t>
         </is>
       </c>
     </row>
@@ -517,17 +528,22 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>iQ Native</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>iQ MCP</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Total Questions</t>
         </is>
@@ -544,13 +560,18 @@
           <t>suraj@equipfoods.com</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="F5" s="7" t="n">
         <v>14</v>
       </c>
     </row>
@@ -565,13 +586,18 @@
           <t>deanna@equipfoods.com</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="F6" s="7" t="n">
         <v>14</v>
       </c>
     </row>
@@ -586,178 +612,247 @@
           <t>alexb@equipfoods.com</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="E7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>3 users</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="8" t="inlineStr"/>
+      <c r="D8" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>None of these users were active in the last 30 / 14 / 7 days — recent EquipFoods volume is all Equipfoods Pulse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>These are all-time figures. None of these three users were active in the last 30 days, last 14 days, or last 7 days — their activity sits entirely outside those windows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Excludes the Equipfoods Pulse account (analytics.saras@equipfoods.com), which is the only EquipFoods account with activity in the last 30 / 14 / 7 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>TrueSeaMoss (TSM)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>iQ adoption by user — all-time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Time period: ALL TIME (all available data — dashboard range May 3, 2026 – Sep 11, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>iQ Native</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>iQ MCP</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Total Questions</t>
         </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>TrueSeaMossProd Iq</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr"/>
-      <c r="C16" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>54</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Analytics Saras</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>93</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>gega trueseamoss</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>11</v>
+          <t>TrueSeaMossProd Iq</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>email not shown in dashboard</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>p.josanu</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="6" t="n">
+          <t>Analytics Saras</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>analyticssaras@trueseamoss.com</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>gega trueseamoss</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>gega@trueseamoss.com</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>p josanu</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>p.josanu@trueseamoss.com</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Multi</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="E21" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="6" t="n">
+      <c r="F21" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>4 users</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C22" s="8" t="inlineStr"/>
+      <c r="D22" s="9" t="n">
         <v>102</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="E22" s="9" t="n">
         <v>113</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="F22" s="9" t="n">
         <v>215</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Last 7 days: Analytics Saras only (3 questions, all iQ MCP). TrueSeaMossProd Iq, gega and p.josanu are inactive in that window.</t>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>These are all-time figures. Recent windows are much smaller: last 30 days = 13 questions / 3 users, last 14 days = 7 questions / 2 users, last 7 days = 3 questions / 1 user (Analytics Saras, all via iQ MCP).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>gega trueseamoss and TrueSeaMossProd Iq were active in the 14- and 30-day windows but not in the last 7 days; p josanu is all-time only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>The dashboard's external-customers-only view lists 3 TSM users (106 questions) and does not show TrueSeaMossProd Iq or its email; that account's 109 questions are included above to reach the 215 all-time total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclude Analytics Saras and TrueSeaMossProd Iq from TSM table
TrueSeaMoss now lists only gega trueseamoss and p josanu (2 users,
13 questions all-time), with footnotes updated accordingly.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxMtvSYX4QyFmV6dcFDu1y
</commit_message>
<xml_diff>
--- a/iq_adoption_equipfoods_tsm.xlsx
+++ b/iq_adoption_equipfoods_tsm.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -712,38 +712,38 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TrueSeaMossProd Iq</t>
+          <t>gega trueseamoss</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>email not shown in dashboard</t>
+          <t>gega@trueseamoss.com</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Multi</t>
+          <t>Native</t>
         </is>
       </c>
       <c r="D18" s="7" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Analytics Saras</t>
+          <t>p josanu</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>analyticssaras@trueseamoss.com</t>
+          <t>p.josanu@trueseamoss.com</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -752,107 +752,55 @@
         </is>
       </c>
       <c r="D19" s="7" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>93</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>gega trueseamoss</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>gega@trueseamoss.com</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Native</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>p josanu</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>p.josanu@trueseamoss.com</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Multi</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>2 users</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr"/>
+      <c r="D20" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="7" t="n">
-        <v>2</v>
+      <c r="F20" s="9" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>4 users</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr"/>
-      <c r="D22" s="9" t="n">
-        <v>102</v>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>113</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>215</v>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>These are all-time figures. Excludes Analytics Saras (analyticssaras@trueseamoss.com) and TrueSeaMossProd Iq.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>gega trueseamoss was active in the last 30 and 14 days (3 questions, iQ Native) but not in the last 7 days. p josanu shows all-time activity only.</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>These are all-time figures. Recent windows are much smaller: last 30 days = 13 questions / 3 users, last 14 days = 7 questions / 2 users, last 7 days = 3 questions / 1 user (Analytics Saras, all via iQ MCP).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>gega trueseamoss and TrueSeaMossProd Iq were active in the 14- and 30-day windows but not in the last 7 days; p josanu is all-time only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>The dashboard's external-customers-only view lists 3 TSM users (106 questions) and does not show TrueSeaMossProd Iq or its email; that account's 109 questions are included above to reach the 215 all-time total.</t>
+          <t>Neither of these two users was active in the last 7 days.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add last-30-day and last-14-day sections for TrueSeaMoss
TSM is now split into All Time, Last 30 Days and Last 14 Days sections,
each excluding Analytics Saras and TrueSeaMossProd Iq, with notes on the
excluded volume per window.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxMtvSYX4QyFmV6dcFDu1y
</commit_message>
<xml_diff>
--- a/iq_adoption_equipfoods_tsm.xlsx
+++ b/iq_adoption_equipfoods_tsm.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0;&quot;—&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +31,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="002D2D2D"/>
-      <sz val="13"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002D2D2D"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -105,28 +111,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -510,297 +520,527 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>All Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Time period: ALL TIME (all available data — dashboard range May 3, 2026 – Sep 11, 2026)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>iQ Native</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>iQ MCP</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Total Questions</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Suraj Dave</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>suraj@equipfoods.com</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Native</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F7" s="8" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Deanna Eng</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>deanna@equipfoods.com</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Native</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F8" s="8" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Alex Beshansky</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>alexb@equipfoods.com</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Native</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F9" s="8" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>3 users</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="9" t="n">
+      <c r="C10" s="10" t="inlineStr"/>
+      <c r="D10" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F10" s="11" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>These are all-time figures. None of these three users were active in the last 30 days, last 14 days, or last 7 days — their activity sits entirely outside those windows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>These are all-time figures. None of these three users were active in the last 30 days, last 14 days, or last 7 days — their activity sits entirely outside those windows, so there is no separate 30-day or 14-day section for EquipFoods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Excludes the Equipfoods Pulse account (analytics.saras@equipfoods.com), which is the only EquipFoods account with activity in the last 30 / 14 / 7 days.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>TrueSeaMoss (TSM)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>All sections below exclude Analytics Saras (analyticssaras@trueseamoss.com) and TrueSeaMossProd Iq.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>All Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Time period: ALL TIME (all available data — dashboard range May 3, 2026 – Sep 11, 2026)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>User</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>iQ Native</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>iQ MCP</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Total Questions</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>gega trueseamoss</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>gega@trueseamoss.com</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Native</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F23" s="8" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>p josanu</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>p.josanu@trueseamoss.com</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Multi</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D24" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="E24" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="7" t="n">
+      <c r="F24" s="8" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>2 users</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="9" t="n">
+      <c r="C25" s="10" t="inlineStr"/>
+      <c r="D25" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E25" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="F25" s="11" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>These are all-time figures. Excludes Analytics Saras (analyticssaras@trueseamoss.com) and TrueSeaMossProd Iq.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>gega trueseamoss was active in the last 30 and 14 days (3 questions, iQ Native) but not in the last 7 days. p josanu shows all-time activity only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Neither of these two users was active in the last 7 days.</t>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Full TSM all-time volume is 215 questions / 4 users; the two excluded accounts account for 202 of those questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Last 30 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Time period: LAST 30 DAYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>iQ Native</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>iQ MCP</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>gega trueseamoss</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>gega@trueseamoss.com</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>1 user</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr"/>
+      <c r="D34" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>p josanu had no activity in this window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Full TSM last-30-day volume is 13 questions / 3 users — the other 10 questions belong to the two excluded accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Last 14 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Time period: LAST 14 DAYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>iQ Native</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>iQ MCP</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Total Questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>gega trueseamoss</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>gega@trueseamoss.com</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>1 user</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr"/>
+      <c r="D44" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>Identical to the last-30-day figures — all of gega's recent activity falls inside the last 14 days. p josanu had no activity in this window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Full TSM last-14-day volume is 7 questions / 2 users — the other 4 belong to Analytics Saras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>Last 7 days is not shown because it would be empty: the only TSM user active in that window was Analytics Saras (3 questions, iQ MCP), which is excluded here.</t>
         </is>
       </c>
     </row>

</xml_diff>